<commit_message>
Published state of ETDataset for deploy 2026-05
</commit_message>
<xml_diff>
--- a/pipelines/Deferred work tracking.xlsx
+++ b/pipelines/Deferred work tracking.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10209"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/koenvanbemmelen/work/etdataset/pipelines/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyradehaan/github/etdataset/pipelines/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE0325E-8008-184A-AFAA-78EE9346E7BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8C7D8DA-B130-E54D-AF5D-31D8E0177256}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="500" windowWidth="37320" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11340" yWindow="-28800" windowWidth="51200" windowHeight="28800" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Instructions" sheetId="2" r:id="rId1"/>
@@ -33,8 +33,26 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={4C963840-5CAC-894A-A497-054BC6085AFE}</author>
+  </authors>
+  <commentList>
+    <comment ref="B42" authorId="0" shapeId="0" xr:uid="{4C963840-5CAC-894A-A497-054BC6085AFE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Requires clarification. What does this mean?</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="197" uniqueCount="111">
   <si>
     <t>Pipeline Step</t>
   </si>
@@ -46,9 +64,6 @@
   </si>
   <si>
     <t>METADATA</t>
-  </si>
-  <si>
-    <t>Deploy</t>
   </si>
   <si>
     <t>Date processed</t>
@@ -331,13 +346,71 @@
     <t>Add clarifications in the optional grey fields.</t>
   </si>
   <si>
-    <t>Ask Kas Kranenburg or Koen van Bemmelen for help when in doubt.</t>
-  </si>
-  <si>
     <t>Status updates</t>
   </si>
   <si>
     <t>v1.0 of this deferred work tracking document created. The 'Quick fixes' in the Post-processing notebook still need to be created; not in use yet.</t>
+  </si>
+  <si>
+    <t>Update biogenic waste inputs</t>
+  </si>
+  <si>
+    <t>Kas Kranenburg, Kyra de Haan &amp; Koen van Bemmelen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">energy_distribution_biogenic_waste_energy_distribution_waste_mix_child_share --&gt; input_percentage_of_biogenic_waste_energy_distribution_waste_mix
+energy_distribution_non_biogenic_waste_energy_distribution_waste_mix_child_share --&gt; input_percentage_of_non_biogenic_waste_energy_distribution_waste_mix </t>
+  </si>
+  <si>
+    <t>Checked: no ETLocal keys rely on this input. Updated YAML is necessary to fill the ETLocal template with data from the national dataset in the preprocessing notebook</t>
+  </si>
+  <si>
+    <t>New keys need to be included in the ETLocal template</t>
+  </si>
+  <si>
+    <t>These inputs are not used in any of the sector notebooks</t>
+  </si>
+  <si>
+    <t>If the Extract and preprocess notebook is run, both data.csv and commits.yaml should be updated accordingly in this notebook. Running this notebook has not been done yet</t>
+  </si>
+  <si>
+    <t>Separate ETLocal data migration has been performed for this update</t>
+  </si>
+  <si>
+    <t>Minor update. Postponed so that it can be bundled with future updates.</t>
+  </si>
+  <si>
+    <t>Rename gas power plant keys</t>
+  </si>
+  <si>
+    <t>Ask Koen van Bemmelen for help when in doubt.</t>
+  </si>
+  <si>
+    <t>Kyra de Haan</t>
+  </si>
+  <si>
+    <t>energy_power_combined_cycle_network_gas_full_load_hours --&gt; input_energy_power_combined_cycle_network_gas_full_load_hours
+energy_power_turbine_network_gas_full_load_hours --&gt; input_energy_power_turbine_network_gas_full_load_hours</t>
+  </si>
+  <si>
+    <t>YAMLs should be renamed for:
+- energy_power_combined_cycle_network_gas_full_load_hours
+- energy_power_turbine_network_gas_full_load_hours</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Deploy tag</t>
+  </si>
+  <si>
+    <t>Deploy date</t>
+  </si>
+  <si>
+    <t>2026-04</t>
+  </si>
+  <si>
+    <t>2025.12</t>
   </si>
 </sst>
 </file>
@@ -748,14 +821,14 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="8" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="9" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="8" fillId="9" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="14" fontId="7" fillId="9" borderId="6" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -764,7 +837,207 @@
     <cellStyle name="Normal 2" xfId="3" xr:uid="{04AF4DDF-7DD8-594B-B003-C9E26A2A90F1}"/>
     <cellStyle name="Per cent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="8">
+  <dxfs count="28">
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.14996795556505021"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.14996795556505021"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.14996795556505021"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.14996795556505021"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.14996795556505021"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF006100"/>
@@ -861,6 +1134,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Koen van Bemmelen" id="{4BD46035-F20E-234D-B4C2-573DB9D4CD56}" userId="S::koen.vanbemmelen@quintel.com::3e1b4bb7-59fe-4b2c-b92b-6e594f408859" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1146,6 +1425,14 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="B42" dT="2026-05-08T14:36:39.83" personId="{4BD46035-F20E-234D-B4C2-573DB9D4CD56}" id="{4C963840-5CAC-894A-A497-054BC6085AFE}">
+    <text>Requires clarification. What does this mean?</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{51D7A9D5-C897-0344-9111-224DD7C73994}">
   <sheetPr>
@@ -1164,7 +1451,7 @@
   <sheetData>
     <row r="3" spans="2:8">
       <c r="B3" s="13" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C3" s="14"/>
       <c r="D3" s="15"/>
@@ -1185,7 +1472,7 @@
     <row r="5" spans="2:8">
       <c r="B5" s="19"/>
       <c r="C5" s="24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D5" s="20"/>
       <c r="E5" s="20"/>
@@ -1193,10 +1480,10 @@
       <c r="G5" s="20"/>
       <c r="H5" s="21"/>
     </row>
-    <row r="6" spans="2:8" ht="28">
+    <row r="6" spans="2:8">
       <c r="B6" s="22"/>
       <c r="C6" s="25" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D6" s="23"/>
       <c r="E6" s="23"/>
@@ -1207,7 +1494,7 @@
     <row r="7" spans="2:8">
       <c r="B7" s="22"/>
       <c r="C7" s="25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D7" s="23"/>
       <c r="E7" s="23"/>
@@ -1227,7 +1514,7 @@
     <row r="9" spans="2:8">
       <c r="B9" s="19"/>
       <c r="C9" s="24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D9" s="26"/>
       <c r="E9" s="27"/>
@@ -1235,10 +1522,10 @@
       <c r="G9" s="20"/>
       <c r="H9" s="21"/>
     </row>
-    <row r="10" spans="2:8" ht="28">
+    <row r="10" spans="2:8">
       <c r="B10" s="19"/>
       <c r="C10" s="25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D10" s="26"/>
       <c r="E10" s="28"/>
@@ -1267,7 +1554,7 @@
     <row r="13" spans="2:8">
       <c r="B13" s="19"/>
       <c r="C13" s="23" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D13" s="27"/>
       <c r="E13" s="27"/>
@@ -1278,7 +1565,7 @@
     <row r="14" spans="2:8">
       <c r="B14" s="19"/>
       <c r="C14" s="20" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D14" s="20"/>
       <c r="E14" s="20"/>
@@ -1287,11 +1574,11 @@
       <c r="H14" s="21"/>
     </row>
     <row r="15" spans="2:8">
-      <c r="B15" s="59" t="s">
+      <c r="B15" s="58" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="25" t="s">
         <v>85</v>
-      </c>
-      <c r="C15" s="25" t="s">
-        <v>86</v>
       </c>
       <c r="D15" s="20"/>
       <c r="E15" s="27"/>
@@ -1300,11 +1587,11 @@
       <c r="H15" s="21"/>
     </row>
     <row r="16" spans="2:8">
-      <c r="B16" s="59" t="s">
-        <v>87</v>
+      <c r="B16" s="58" t="s">
+        <v>86</v>
       </c>
       <c r="C16" s="30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D16" s="20"/>
       <c r="E16" s="31"/>
@@ -1313,11 +1600,11 @@
       <c r="H16" s="21"/>
     </row>
     <row r="17" spans="2:8">
-      <c r="B17" s="59" t="s">
-        <v>88</v>
+      <c r="B17" s="58" t="s">
+        <v>87</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D17" s="28"/>
       <c r="E17" s="20"/>
@@ -1326,7 +1613,7 @@
       <c r="H17" s="21"/>
     </row>
     <row r="18" spans="2:8">
-      <c r="B18" s="59"/>
+      <c r="B18" s="58"/>
       <c r="C18" s="30"/>
       <c r="D18" s="20"/>
       <c r="E18" s="32"/>
@@ -1335,9 +1622,9 @@
       <c r="H18" s="21"/>
     </row>
     <row r="19" spans="2:8">
-      <c r="B19" s="59"/>
+      <c r="B19" s="58"/>
       <c r="C19" s="30" t="s">
-        <v>91</v>
+        <v>102</v>
       </c>
       <c r="D19" s="20"/>
       <c r="E19" s="31"/>
@@ -1346,7 +1633,7 @@
       <c r="H19" s="21"/>
     </row>
     <row r="20" spans="2:8">
-      <c r="B20" s="59"/>
+      <c r="B20" s="58"/>
       <c r="C20" s="20"/>
       <c r="D20" s="20"/>
       <c r="E20" s="20"/>
@@ -1355,9 +1642,9 @@
       <c r="H20" s="21"/>
     </row>
     <row r="21" spans="2:8">
-      <c r="B21" s="60"/>
+      <c r="B21" s="59"/>
       <c r="C21" s="24" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D21" s="20"/>
       <c r="E21" s="20"/>
@@ -1366,11 +1653,11 @@
       <c r="H21" s="21"/>
     </row>
     <row r="22" spans="2:8">
-      <c r="B22" s="60">
+      <c r="B22" s="59">
         <v>45985</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="D22" s="24"/>
       <c r="E22" s="20"/>
@@ -1978,19 +2265,19 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="0.39997558519241921"/>
   </sheetPr>
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:F64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="55.1640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="40" customWidth="1"/>
+    <col min="3" max="6" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16">
+    <row r="1" spans="1:6" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1998,613 +2285,944 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="20" customHeight="1">
+    <row r="2" spans="1:6" ht="20" customHeight="1">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
         <v>3</v>
       </c>
       <c r="C2" s="2"/>
-      <c r="D2" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="20" customHeight="1">
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="20" customHeight="1">
       <c r="A3" s="3" t="s">
-        <v>4</v>
+        <v>107</v>
       </c>
       <c r="B3" s="3"/>
-      <c r="C3" s="8">
-        <v>46002</v>
-      </c>
-      <c r="D3" s="8"/>
-    </row>
-    <row r="4" spans="1:4" ht="20" customHeight="1">
+      <c r="C3" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="60" t="s">
+        <v>110</v>
+      </c>
+      <c r="E3" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="F3" s="8"/>
+    </row>
+    <row r="4" spans="1:6" ht="20" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>5</v>
+        <v>108</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="8">
+        <v>46003</v>
+      </c>
+      <c r="D4" s="8">
+        <v>46003</v>
+      </c>
+      <c r="E4" s="8">
+        <v>46142</v>
+      </c>
+      <c r="F4" s="8"/>
+    </row>
+    <row r="5" spans="1:6" ht="20" customHeight="1">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="8">
         <v>45982</v>
       </c>
-      <c r="D4" s="8"/>
-    </row>
-    <row r="5" spans="1:4" ht="20" customHeight="1">
-      <c r="A5" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5" s="3"/>
-      <c r="C5" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D5" s="4"/>
-    </row>
-    <row r="6" spans="1:4" ht="20" customHeight="1">
-      <c r="A6" s="3"/>
+      <c r="D5" s="8">
+        <v>45989</v>
+      </c>
+      <c r="E5" s="8">
+        <v>46149</v>
+      </c>
+      <c r="F5" s="8"/>
+    </row>
+    <row r="6" spans="1:6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>5</v>
+      </c>
       <c r="B6" s="3"/>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-    </row>
-    <row r="7" spans="1:4" ht="20" customHeight="1">
-      <c r="A7" s="5"/>
-      <c r="B7" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="5"/>
-    </row>
-    <row r="8" spans="1:4" ht="20" customHeight="1">
-      <c r="A8" s="3"/>
-      <c r="B8" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="4"/>
-    </row>
-    <row r="9" spans="1:4" ht="20" customHeight="1">
+      <c r="C6" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F6" s="4"/>
+    </row>
+    <row r="7" spans="1:6" ht="20" customHeight="1">
+      <c r="A7" s="3"/>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+    </row>
+    <row r="8" spans="1:6" ht="20" customHeight="1">
+      <c r="A8" s="5"/>
+      <c r="B8" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
+      <c r="F8" s="5"/>
+    </row>
+    <row r="9" spans="1:6" ht="20" customHeight="1">
       <c r="A9" s="3"/>
       <c r="B9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" s="11"/>
-      <c r="D9" s="11"/>
-    </row>
-    <row r="10" spans="1:4" ht="20" customHeight="1">
+        <v>62</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F9" s="4"/>
+    </row>
+    <row r="10" spans="1:6" ht="20" customHeight="1">
       <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="11" spans="1:4" ht="20" customHeight="1">
-      <c r="A11" s="5"/>
-      <c r="B11" s="5" t="s">
+      <c r="B10" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+    </row>
+    <row r="11" spans="1:6" ht="20" customHeight="1">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" ht="20" customHeight="1">
+      <c r="A12" s="5"/>
+      <c r="B12" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
+      <c r="F12" s="5"/>
+    </row>
+    <row r="13" spans="1:6" ht="20" customHeight="1">
+      <c r="A13" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-    </row>
-    <row r="12" spans="1:4" ht="20" customHeight="1">
-      <c r="A12" s="3" t="s">
+      <c r="B13" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="C13" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F13" s="4"/>
+    </row>
+    <row r="14" spans="1:6" ht="20" customHeight="1">
+      <c r="A14" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="B14" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="4"/>
+    </row>
+    <row r="15" spans="1:6" s="10" customFormat="1" ht="144">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>94</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15" s="9"/>
+    </row>
+    <row r="16" spans="1:6" ht="20" customHeight="1">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:6" ht="20" customHeight="1">
+      <c r="A17" s="5"/>
+      <c r="B17" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="C17" s="5"/>
+      <c r="D17" s="5"/>
+      <c r="E17" s="5"/>
+      <c r="F17" s="5"/>
+    </row>
+    <row r="18" spans="1:6" ht="16">
+      <c r="A18" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B18" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F18" s="4"/>
+    </row>
+    <row r="19" spans="1:6" ht="20" customHeight="1">
+      <c r="A19" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B19" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="4"/>
+    </row>
+    <row r="20" spans="1:6" ht="112">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="4"/>
-    </row>
-    <row r="13" spans="1:4" ht="20" customHeight="1">
-      <c r="A13" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D13" s="4"/>
-    </row>
-    <row r="14" spans="1:4" s="10" customFormat="1" ht="64">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>48</v>
-      </c>
-      <c r="D14" s="9"/>
-    </row>
-    <row r="15" spans="1:4" ht="20" customHeight="1">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-    </row>
-    <row r="16" spans="1:4" ht="20" customHeight="1">
-      <c r="A16" s="5"/>
-      <c r="B16" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-    </row>
-    <row r="17" spans="1:4" ht="16">
-      <c r="A17" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D17" s="4"/>
-    </row>
-    <row r="18" spans="1:4" ht="20" customHeight="1">
-      <c r="A18" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="B18" s="3" t="s">
+      <c r="D20" s="9" t="s">
+        <v>95</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F20" s="9"/>
+    </row>
+    <row r="21" spans="1:6" ht="20" customHeight="1">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+    </row>
+    <row r="22" spans="1:6" ht="20" customHeight="1">
+      <c r="A22" s="5"/>
+      <c r="B22" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D18" s="4"/>
-    </row>
-    <row r="19" spans="1:4" ht="96">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C19" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="9"/>
-    </row>
-    <row r="20" spans="1:4" ht="20" customHeight="1">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-    </row>
-    <row r="21" spans="1:4" ht="20" customHeight="1">
-      <c r="A21" s="5"/>
-      <c r="B21" s="5" t="s">
+      <c r="C22" s="5"/>
+      <c r="D22" s="5"/>
+      <c r="E22" s="5"/>
+      <c r="F22" s="5"/>
+    </row>
+    <row r="23" spans="1:6" ht="20" customHeight="1">
+      <c r="A23" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C21" s="5"/>
-      <c r="D21" s="5"/>
-    </row>
-    <row r="22" spans="1:4" ht="20" customHeight="1">
-      <c r="A22" s="3" t="s">
+      <c r="B23" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B22" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="C22" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" s="4"/>
-    </row>
-    <row r="23" spans="1:4" ht="20" customHeight="1">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="C23" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="D23" s="4"/>
-    </row>
-    <row r="24" spans="1:4" ht="66" customHeight="1">
+        <v>45</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F23" s="4"/>
+    </row>
+    <row r="24" spans="1:6" ht="20" customHeight="1">
       <c r="A24" s="3"/>
       <c r="B24" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>64</v>
-      </c>
-      <c r="D24" s="9"/>
-    </row>
-    <row r="25" spans="1:4" ht="20" customHeight="1">
+        <v>48</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F24" s="4"/>
+    </row>
+    <row r="25" spans="1:6" ht="66" customHeight="1">
       <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-    </row>
-    <row r="26" spans="1:4" ht="20" customHeight="1">
-      <c r="A26" s="5"/>
-      <c r="B26" s="5" t="s">
+      <c r="B25" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C25" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>96</v>
+      </c>
+      <c r="F25" s="9"/>
+    </row>
+    <row r="26" spans="1:6" ht="20" customHeight="1">
+      <c r="A26" s="3"/>
+      <c r="B26" s="3"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+    </row>
+    <row r="27" spans="1:6" ht="20" customHeight="1">
+      <c r="A27" s="5"/>
+      <c r="B27" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="C27" s="5"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+    </row>
+    <row r="28" spans="1:6" ht="20" customHeight="1">
+      <c r="A28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C26" s="5"/>
-      <c r="D26" s="5"/>
-    </row>
-    <row r="27" spans="1:4" ht="20" customHeight="1">
-      <c r="A27" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="C27" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D27" s="4"/>
-    </row>
-    <row r="28" spans="1:4" ht="20" customHeight="1">
-      <c r="A28" s="3"/>
       <c r="B28" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D28" s="4"/>
-    </row>
-    <row r="29" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F28" s="4"/>
+    </row>
+    <row r="29" spans="1:6" ht="20" customHeight="1">
       <c r="A29" s="3"/>
       <c r="B29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D29" s="4"/>
-    </row>
-    <row r="30" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F29" s="4"/>
+    </row>
+    <row r="30" spans="1:6" ht="20" customHeight="1">
       <c r="A30" s="3"/>
       <c r="B30" s="3" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D30" s="4"/>
-    </row>
-    <row r="31" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F30" s="4"/>
+    </row>
+    <row r="31" spans="1:6" ht="20" customHeight="1">
       <c r="A31" s="3"/>
       <c r="B31" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D31" s="4"/>
-    </row>
-    <row r="32" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" s="4"/>
+    </row>
+    <row r="32" spans="1:6" ht="20" customHeight="1">
       <c r="A32" s="3"/>
       <c r="B32" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="4"/>
-    </row>
-    <row r="33" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F32" s="4"/>
+    </row>
+    <row r="33" spans="1:6" ht="20" customHeight="1">
       <c r="A33" s="3"/>
       <c r="B33" s="3" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" s="4"/>
-    </row>
-    <row r="34" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F33" s="4"/>
+    </row>
+    <row r="34" spans="1:6" ht="20" customHeight="1">
       <c r="A34" s="3"/>
       <c r="B34" s="3" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="4"/>
-    </row>
-    <row r="35" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F34" s="4"/>
+    </row>
+    <row r="35" spans="1:6" ht="20" customHeight="1">
       <c r="A35" s="3"/>
       <c r="B35" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D35" s="4"/>
-    </row>
-    <row r="36" spans="1:4" ht="20" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F35" s="4"/>
+    </row>
+    <row r="36" spans="1:6" ht="20" customHeight="1">
       <c r="A36" s="3"/>
       <c r="B36" s="3" t="s">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D36" s="4"/>
-    </row>
-    <row r="37" spans="1:4" ht="60" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F36" s="4"/>
+    </row>
+    <row r="37" spans="1:6" ht="20" customHeight="1">
       <c r="A37" s="3"/>
       <c r="B37" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F37" s="4"/>
+    </row>
+    <row r="38" spans="1:6" ht="60" customHeight="1">
+      <c r="A38" s="3"/>
+      <c r="B38" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C38" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D38" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="E38" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="F38" s="9"/>
+    </row>
+    <row r="39" spans="1:6" ht="20" customHeight="1">
+      <c r="A39" s="3"/>
+      <c r="B39" s="3"/>
+      <c r="C39" s="3"/>
+      <c r="D39" s="3"/>
+      <c r="E39" s="3"/>
+      <c r="F39" s="3"/>
+    </row>
+    <row r="40" spans="1:6" ht="20" customHeight="1">
+      <c r="A40" s="5"/>
+      <c r="B40" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D37" s="9"/>
-    </row>
-    <row r="38" spans="1:4" ht="20" customHeight="1">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-    </row>
-    <row r="39" spans="1:4" ht="20" customHeight="1">
-      <c r="A39" s="5"/>
-      <c r="B39" s="5" t="s">
+      <c r="C40" s="5"/>
+      <c r="D40" s="5"/>
+      <c r="E40" s="5"/>
+      <c r="F40" s="5"/>
+    </row>
+    <row r="41" spans="1:6" ht="20" customHeight="1">
+      <c r="A41" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C39" s="5"/>
-      <c r="D39" s="5"/>
-    </row>
-    <row r="40" spans="1:4" ht="20" customHeight="1">
-      <c r="A40" s="3" t="s">
+      <c r="B41" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B40" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D40" s="4"/>
-    </row>
-    <row r="41" spans="1:4" ht="20" customHeight="1">
-      <c r="A41" s="3"/>
-      <c r="B41" s="3" t="s">
-        <v>61</v>
-      </c>
       <c r="C41" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D41" s="4"/>
-    </row>
-    <row r="42" spans="1:4" ht="56" customHeight="1">
+        <v>11</v>
+      </c>
+      <c r="D41" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E41" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F41" s="4"/>
+    </row>
+    <row r="42" spans="1:6" ht="20" customHeight="1">
       <c r="A42" s="3"/>
       <c r="B42" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="D42" s="9"/>
-    </row>
-    <row r="43" spans="1:4" ht="20" customHeight="1">
+        <v>60</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D42" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="F42" s="4"/>
+    </row>
+    <row r="43" spans="1:6" ht="69" customHeight="1">
       <c r="A43" s="3"/>
-      <c r="B43" s="3"/>
-      <c r="C43" s="3"/>
-      <c r="D43" s="3"/>
-    </row>
-    <row r="44" spans="1:4" ht="20" customHeight="1">
-      <c r="A44" s="5"/>
-      <c r="B44" s="5" t="s">
+      <c r="B43" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C43" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D43" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="F43" s="9"/>
+    </row>
+    <row r="44" spans="1:6" ht="20" customHeight="1">
+      <c r="A44" s="3"/>
+      <c r="B44" s="3"/>
+      <c r="C44" s="3"/>
+      <c r="D44" s="3"/>
+      <c r="E44" s="3"/>
+      <c r="F44" s="3"/>
+    </row>
+    <row r="45" spans="1:6" ht="20" customHeight="1">
+      <c r="A45" s="5"/>
+      <c r="B45" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="C45" s="5"/>
+      <c r="D45" s="5"/>
+      <c r="E45" s="5"/>
+      <c r="F45" s="5"/>
+    </row>
+    <row r="46" spans="1:6" ht="20" customHeight="1">
+      <c r="A46" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E46" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F46" s="4"/>
+    </row>
+    <row r="47" spans="1:6" ht="20" customHeight="1">
+      <c r="A47" s="3"/>
+      <c r="B47" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E47" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F47" s="4"/>
+    </row>
+    <row r="48" spans="1:6" ht="20" customHeight="1">
+      <c r="A48" s="3"/>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+      <c r="E48" s="3"/>
+      <c r="F48" s="3"/>
+    </row>
+    <row r="49" spans="1:6" ht="20" customHeight="1">
+      <c r="A49" s="5"/>
+      <c r="B49" s="5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C49" s="5"/>
+      <c r="D49" s="5"/>
+      <c r="E49" s="5"/>
+      <c r="F49" s="5"/>
+    </row>
+    <row r="50" spans="1:6" ht="20" customHeight="1">
+      <c r="A50" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B50" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C50" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D50" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="4"/>
+    </row>
+    <row r="51" spans="1:6" ht="44" customHeight="1">
+      <c r="A51" s="3"/>
+      <c r="B51" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C51" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="D51" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="E51" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="F51" s="9"/>
+    </row>
+    <row r="52" spans="1:6" ht="20" customHeight="1">
+      <c r="A52" s="3"/>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+      <c r="D52" s="3"/>
+      <c r="E52" s="3"/>
+      <c r="F52" s="3"/>
+    </row>
+    <row r="53" spans="1:6" ht="20" customHeight="1">
+      <c r="A53" s="5"/>
+      <c r="B53" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C53" s="5"/>
+      <c r="D53" s="5"/>
+      <c r="E53" s="5"/>
+      <c r="F53" s="5"/>
+    </row>
+    <row r="54" spans="1:6" ht="48">
+      <c r="A54" s="12" t="s">
         <v>65</v>
       </c>
-      <c r="C44" s="5"/>
-      <c r="D44" s="5"/>
-    </row>
-    <row r="45" spans="1:4" ht="20" customHeight="1">
-      <c r="A45" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="B45" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D45" s="4"/>
-    </row>
-    <row r="46" spans="1:4" ht="20" customHeight="1">
-      <c r="A46" s="3"/>
-      <c r="B46" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C46" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D46" s="4"/>
-    </row>
-    <row r="47" spans="1:4" ht="20" customHeight="1">
-      <c r="A47" s="3"/>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-    </row>
-    <row r="48" spans="1:4" ht="20" customHeight="1">
-      <c r="A48" s="5"/>
-      <c r="B48" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="C48" s="5"/>
-      <c r="D48" s="5"/>
-    </row>
-    <row r="49" spans="1:4" ht="20" customHeight="1">
-      <c r="A49" s="12" t="s">
+      <c r="B54" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C54" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D54" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="E54" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="F54" s="4"/>
+    </row>
+    <row r="55" spans="1:6" ht="60" customHeight="1">
+      <c r="A55" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="B55" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C55" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D55" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E55" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F55" s="4"/>
+    </row>
+    <row r="56" spans="1:6" ht="20" customHeight="1">
+      <c r="A56" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B56" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C56" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D56" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E56" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="F56" s="4"/>
+    </row>
+    <row r="57" spans="1:6" ht="20" customHeight="1">
+      <c r="A57" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B57" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="C57" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="D57" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="E57" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F57" s="4"/>
+    </row>
+    <row r="59" spans="1:6" ht="20" customHeight="1">
+      <c r="A59" s="6"/>
+      <c r="B59" s="6" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="20" customHeight="1">
+      <c r="A60" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B60" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" ht="20" customHeight="1">
+      <c r="A61" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="B61" s="7" t="s">
         <v>77</v>
       </c>
-      <c r="B49" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="C49" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D49" s="4"/>
-    </row>
-    <row r="50" spans="1:4" ht="20" customHeight="1">
-      <c r="A50" s="3"/>
-      <c r="B50" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="C50" s="9"/>
-      <c r="D50" s="9"/>
-    </row>
-    <row r="51" spans="1:4" ht="20" customHeight="1">
-      <c r="A51" s="3"/>
-      <c r="B51" s="3"/>
-      <c r="C51" s="58"/>
-      <c r="D51" s="58"/>
-    </row>
-    <row r="52" spans="1:4" ht="20" customHeight="1">
-      <c r="A52" s="5"/>
-      <c r="B52" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="C52" s="5"/>
-      <c r="D52" s="5"/>
-    </row>
-    <row r="53" spans="1:4" ht="48">
-      <c r="A53" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B53" s="12" t="s">
-        <v>67</v>
-      </c>
-      <c r="C53" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D53" s="4"/>
-    </row>
-    <row r="54" spans="1:4" ht="60" customHeight="1">
-      <c r="A54" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="B54" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="C54" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="D54" s="4"/>
-    </row>
-    <row r="55" spans="1:4" ht="20" customHeight="1">
-      <c r="A55" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="B55" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C55" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="D55" s="4"/>
-    </row>
-    <row r="56" spans="1:4" ht="20" customHeight="1">
-      <c r="A56" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="B56" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="C56" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D56" s="4"/>
-    </row>
-    <row r="58" spans="1:4" ht="20" customHeight="1">
-      <c r="A58" s="6"/>
-      <c r="B58" s="6" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="59" spans="1:4" ht="20" customHeight="1">
-      <c r="A59" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B59" s="7" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="60" spans="1:4" ht="20" customHeight="1">
-      <c r="A60" s="7" t="s">
+    </row>
+    <row r="62" spans="1:6" ht="20" customHeight="1">
+      <c r="A62" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="B62" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B60" s="7" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="61" spans="1:4" ht="20" customHeight="1">
-      <c r="A61" s="7" t="s">
+    </row>
+    <row r="63" spans="1:6" ht="20" customHeight="1">
+      <c r="A63" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="B61" s="7" t="s">
+      <c r="B63" s="7" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="20" customHeight="1">
-      <c r="A62" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="B62" s="7" t="s">
+    <row r="64" spans="1:6" ht="20" customHeight="1">
+      <c r="A64" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B64" s="7" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="20" customHeight="1">
-      <c r="A63" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B63" s="7" t="s">
-        <v>42</v>
-      </c>
-    </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B27:B36">
-    <sortCondition ref="B36"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B28:B37">
+    <sortCondition ref="B37"/>
   </sortState>
-  <conditionalFormatting sqref="C1:C7 C51:C1048576 C49:D50 C9:C48">
-    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="n/a">
+  <conditionalFormatting sqref="C1:C2 C4:C1048576">
+    <cfRule type="containsText" dxfId="27" priority="33" operator="containsText" text="n/a">
       <formula>NOT(ISERROR(SEARCH("n/a",C1)))</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="6" priority="6" stopIfTrue="1" operator="endsWith" text="x">
+    <cfRule type="endsWith" dxfId="26" priority="34" stopIfTrue="1" operator="endsWith" text="x">
       <formula>RIGHT(C1,LEN("x"))="x"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="5" priority="7" operator="endsWith" text="!">
+    <cfRule type="endsWith" dxfId="25" priority="35" operator="endsWith" text="!">
       <formula>RIGHT(C1,LEN("!"))="!"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="4" priority="8" operator="endsWith" text="v">
+    <cfRule type="endsWith" dxfId="24" priority="36" operator="endsWith" text="v">
       <formula>RIGHT(C1,LEN("v"))="v"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D7 C8:D8 D9:D48 D51:D56">
-    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="n/a">
+  <conditionalFormatting sqref="D5:F18 E4:F4 D20:F57 D19 F19">
+    <cfRule type="containsText" dxfId="23" priority="17" operator="containsText" text="n/a">
+      <formula>NOT(ISERROR(SEARCH("n/a",D4)))</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="22" priority="18" stopIfTrue="1" operator="endsWith" text="x">
+      <formula>RIGHT(D4,LEN("x"))="x"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="21" priority="19" operator="endsWith" text="!">
+      <formula>RIGHT(D4,LEN("!"))="!"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="20" priority="20" operator="endsWith" text="v">
+      <formula>RIGHT(D4,LEN("v"))="v"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3:F3">
+    <cfRule type="containsText" dxfId="19" priority="13" operator="containsText" text="n/a">
+      <formula>NOT(ISERROR(SEARCH("n/a",E3)))</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="18" priority="14" stopIfTrue="1" operator="endsWith" text="x">
+      <formula>RIGHT(E3,LEN("x"))="x"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="17" priority="15" operator="endsWith" text="!">
+      <formula>RIGHT(E3,LEN("!"))="!"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="16" priority="16" operator="endsWith" text="v">
+      <formula>RIGHT(E3,LEN("v"))="v"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D4">
+    <cfRule type="containsText" dxfId="15" priority="9" operator="containsText" text="n/a">
+      <formula>NOT(ISERROR(SEARCH("n/a",D4)))</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="14" priority="10" stopIfTrue="1" operator="endsWith" text="x">
+      <formula>RIGHT(D4,LEN("x"))="x"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="13" priority="11" operator="endsWith" text="!">
+      <formula>RIGHT(D4,LEN("!"))="!"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="12" priority="12" operator="endsWith" text="v">
+      <formula>RIGHT(D4,LEN("v"))="v"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:D3">
+    <cfRule type="containsText" dxfId="7" priority="5" operator="containsText" text="n/a">
       <formula>NOT(ISERROR(SEARCH("n/a",C3)))</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="2" priority="2" stopIfTrue="1" operator="endsWith" text="x">
+    <cfRule type="endsWith" dxfId="6" priority="6" stopIfTrue="1" operator="endsWith" text="x">
       <formula>RIGHT(C3,LEN("x"))="x"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="1" priority="3" operator="endsWith" text="!">
+    <cfRule type="endsWith" dxfId="5" priority="7" operator="endsWith" text="!">
       <formula>RIGHT(C3,LEN("!"))="!"</formula>
     </cfRule>
-    <cfRule type="endsWith" dxfId="0" priority="4" operator="endsWith" text="v">
+    <cfRule type="endsWith" dxfId="4" priority="8" operator="endsWith" text="v">
       <formula>RIGHT(C3,LEN("v"))="v"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="E19">
+    <cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="n/a">
+      <formula>NOT(ISERROR(SEARCH("n/a",E19)))</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="2" priority="2" stopIfTrue="1" operator="endsWith" text="x">
+      <formula>RIGHT(E19,LEN("x"))="x"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="1" priority="3" operator="endsWith" text="!">
+      <formula>RIGHT(E19,LEN("!"))="!"</formula>
+    </cfRule>
+    <cfRule type="endsWith" dxfId="0" priority="4" operator="endsWith" text="v">
+      <formula>RIGHT(E19,LEN("v"))="v"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C12:D13 C45:D46 C40:D41 C49:D49 C22:D23 C8:D8 C17:D18 C27:D36" xr:uid="{E66FCAB3-ECA7-C549-86D6-2EAF3DF4A340}">
-      <formula1>$A$59:$A$63</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C9:F9 C50:F50 C28:F37 C13:F14 C46:F47 C23:F24 C41:F42 C18:F19" xr:uid="{E66FCAB3-ECA7-C549-86D6-2EAF3DF4A340}">
+      <formula1>$A$60:$A$64</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>